<commit_message>
add multimodal FM docs and latest review materials
Document the multimodal experiment roadmap and add the newest spreadsheet and presentation assets for review.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/202604 BCSC Innovation Idea Profile - Flow Planner.xlsx
+++ b/202604 BCSC Innovation Idea Profile - Flow Planner.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E52643-7D7D-428C-A8B8-AC69FC090056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A15A80-7222-455C-A2B7-E616019BD174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10830" yWindow="-14805" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -81,116 +81,145 @@
     <t>Input date: 2026/04/09</t>
   </si>
   <si>
-    <t>本项目基于 Flow Planner (NeurIPS 2025) 构建安全自适应的自动驾驶轨迹规划系统。Flow Planner 采用 Flow Matching 生成式框架，仅需 4 步 ODE 求解即可从随机噪声生成未来 8 秒的驾驶轨迹，推理速度比 Diffusion 方法快 5 倍以上，模型仅 14.28M 参数，适合车端部署。_x000D_
-_x000D_
-我们在此基础上提出 5 大创新点：_x000D_
-1) Scene-Adaptive CFG：根据场景风险动态调整 CFG 引导权重，替代全局固定 w=1.8_x000D_
-2) Best-of-N 多候选安全筛选：每步生成 N=5 条候选轨迹，用 5 维安全打分器选最优_x000D_
-3) Risk-Adaptive ODE：风险网络动态控制推理步数（2-6步），平衡安全性与推理效率_x000D_
-4) Safety-Guided Flow Matching：在 ODE 求解过程中注入安全梯度约束，实现主动避碰_x000D_
-5) Goal-Conditioned DPO（借鉴 GoalFlow, CVPR 2025）：通过 goal point conditioning 生成决策级多样性轨迹（左绕/右绕/刹停），构建偏好数据对进行 DPO 训练，从根本上提升模型的安全决策能力</t>
+    <t>Flow Planner 是基于 Flow Matching 的生成式自动驾驶轨迹规划方案（NeurIPS 2025）。与传统 rule-based planner 不同，Flow Planner 通过 4 步 ODE 直接生成未来 8 秒轨迹，参数量仅 14.28M，推理延迟约 20ms，兼顾多模态生成能力与实时性。
+核心问题：基线模型存在"模式坍塌"——多次采样生成的轨迹高度相似，缺乏"左绕/右绕/刹停"等决策级多样性，无法支撑偏好学习。
+核心方案（三阶段递进）：
+1) 意图注入（Goal Conditioning）：借鉴 GoalFlow（CVPR 2025），从 GT 轨迹聚类出 64 个 goal point（4s 终点），通过 AdaLN 注入 decoder，让模型按不同意图生成差异化轨迹
+2) 偏好对齐（Scorer + DPO）：用安全/舒适度评分器构造 chosen/rejected 对，LoRA + DPO 微调，让模型学会公司偏好
+3) 安全落地（Safety-Aware Inference + Domain Transfer）：TTC/DRAC 碰撞校验 + best-of-N 筛选 + 领域迁移，保证部署安全性</t>
   </si>
   <si>
-    <t>1. 安全自适应 Flow Matching 轨迹规划算法库：包含 5 大创新模块（自适应CFG、Best-of-N、风险自适应ODE、安全约束引导、Goal-Conditioned DPO），支持 Python/PyTorch 训练与推理_x000D_
-2. 预训练模型权重：nuPlan 全量数据训练的基线模型 + DPO 微调后的安全增强模型_x000D_
-3. Goal Point 词典：64 个聚类中心的 goal vocabulary (goal_vocab.npy)，支持多模态轨迹生成_x000D_
-4. 端到端自动化 Pipeline：从 goal 聚类 → FM 重训 → 候选生成 → 打分 → DPO 训练 → 评估的一键脚本 (auto_goal_dpo_pipeline.sh)_x000D_
-5. 2 项发明专利申请（自适应 CFG 引导方法 + Safety-Guided Flow Matching 方法）_x000D_
-6. 跨域迁移与三阶段渐进式部署方案文档_x000D_
-7. TensorRT FP16 量化后的车端部署模型（延迟 &lt;50ms）</t>
+    <t>1. 行业趋势：生成式规划已成学术主流方向（NeurIPS/ICLR 2025 多篇相关工作），Tesla FSD v12、Waymo EMMA 均采用端到端生成式架构。图像生成领域 diffusion逐渐被flow matching所替代。不提前布局将失去技术窗口期
+2. 技术成熟：Flow Planner 基线已在 nuPlan benchmark 达到 SOTA 级别（NR=90.43），GoalFlow (CVPR 2025) 验证了 goal conditioning 对 FM 多模态性的有效性——两个关键组件均有学术验证，风险可控
+3. 内部需求：当前 ASW Planning 基于 rule-based 方案，在复杂交互/博弈场景中难以穷举所有策略。生成式方案可作为候选轨迹生成模块，与现有决策层配合
+4. DPO 时机：DPO/RLHF 在 LLM 领域已充分验证，现已开始向自动驾驶规划迁移（TrajHF、MuDi-Pro 等），Flow Planner 的 goal conditioning 恰好解决了 DPO 所需的轨迹多样性前提
+5. 资源窗口：AutoDL 等云 GPU 平台成本持续下降，15 万预算即可覆盖全部算力需求</t>
   </si>
   <si>
-    <t>本项目聚焦于解决生成式轨迹规划从学术到实车部署的三大核心挑战：_x000D_
-_x000D_
-1. 安全性保证：纯模仿学习缺乏对物理安全边界的主动感知。通过 Safety-Guided Flow Matching 在生成过程中注入安全约束，Best-of-N 多候选筛选消灭尾部碰撞事件，Goal-Conditioned DPO 从训练层面对齐安全偏好 - 三重机制形成完整安全闭环。_x000D_
-_x000D_
-2. 场景自适应能力：固定引导权重和推理步数无法适应多变驾驶场景。Scene-Adaptive CFG 和 Risk-Adaptive ODE 让模型根据场景复杂度动态调整行为 - 简单场景快速通过，复杂场景精细规划。_x000D_
-_x000D_
-3. DPO 轨迹多样性：Flow Matching 的 ODE 采样特性导致生成轨迹缺乏决策级多样性（左绕 vs 右绕 vs 刹停），DPO 训练无法进行。借鉴 GoalFlow (CVPR 2025) 的 goal point conditioning，从模型架构层面解决模式坍塌问题，使 DPO 偏好学习首次在 Flow Matching 框架中可行。</t>
+    <t>1. Goal Conditioning 与 Flow Matching 的结合机制：
+   GoalFlow (CVPR 2025) 使用 sinusoidal positional embedding + self-attention 注入 goal；我们基于现有 DiT 架构，改用 goal_proj MLP + AdaLN 注入，改动更小、与现有代码兼容。这种架构级的融合设计需要对 FM 的 ODE 动力学和 DiT 的条件注入机制有深入理解
+2. DPO 在连续轨迹空间的适配：
+   DPO 原设计面向离散 token（LLM），将其迁移到连续轨迹空间需要设计合适的 scorer、采样策略和 preference pair 构造方法。目前业界仅有少数工作（TrajHF、MuDi-Pro）探索这个方向
+3. Safety-Aware Inference 的工程化：
+   将碰撞检测（TTC/DRAC）、adaptive ODE、best-of-N 等机制集成为实时可用的推理 pipeline，需要在安全性和延迟之间做精细平衡
+4. 端到端自动化 Pipeline：
+   从 goal 聚类到 DPO 训练的全流程自动化，包含数据预处理、模型训练、评估的完整闭环，具有较高的工程壁垒
+5. 学术基础：Flow Planner 本身是 NeurIPS 2025 工作，在此基础上的增量创新具有可靠的起点</t>
   </si>
   <si>
-    <t>1. 行业趋势驱动：自动驾驶规划模块正从「写规则」变成「学经验」。Tesla FSD v12、Waymo EMMA 均已转向端到端学习方法。NeurIPS/ICLR 2025 顶会中生成式规划方法已成绝对主流。Flow Planner 以纯学习方法首次突破 nuPlan Val14 90 分大关。_x000D_
-_x000D_
-2. 实车部署刚需：公司 ASW Planning 模块需要从 rule-based 方案向学习型方案演进。现有规则方法在复杂交互场景（抢道、博弈变道、行人避让）中规则写不完，亟需数据驱动方法补充。_x000D_
-_x000D_
-3. 安全合规要求：纯模仿学习在长尾场景中易产生危险决策（如后方快车逼近时仍变道导致碰撞）。实车部署要求规划模块必须有显式安全约束，不能仅依赖隐式学习经验。_x000D_
-_x000D_
-4. 学术前沿对齐：DPO/RLHF 在 LLM 领域已验证有效，将偏好对齐思想引入自动驾驶轨迹规划是学术最前沿方向，目前学界（TrajHF、MuDi-Pro）刚起步探索。</t>
+    <t>1. 跨域迁移模型：nuPlan 预训练 -&gt; 公司数据微调的 Flow Planner 模型 (冻结 Encoder 浅层 + 微调 Decoder)
+2. 车端部署模型：TensorRT FP16 量化后的 .engine 文件, 推理延迟 &lt; 50ms, 满足 10Hz 实时性
+3. 三阶段部署执行：影子模式对比数据 + 场景分级混合部署方案 + 全场景接管方案
+4. 实车验证报告：路口场景闭环测试结果 (碰撞率, TTC 合规率, 舒适度, 通过率)
+5. 2 项发明专利正式提交 (自适应 CFG + Safety-Guided Flow Matching)
+6. 结题报告：完整技术方案、实验数据、部署方案、投入产出分析</t>
   </si>
   <si>
-    <t>1. 安全性提升：Safety-Guided FM + Best-of-N 双重安全机制，碰撞率预期降低 30%+；DPO 训练从根本上改变模型输出分布，主动避开危险轨迹。_x000D_
-_x000D_
-2. 推理效率优势：Flow Matching 4步推理 vs Diffusion 20+步，速度提升 5 倍（~12Hz, 自适应ODE可达 ~25Hz）。模型仅 14.28M 参数 (57MB)，TensorRT FP16 后 &lt;30MB，适配 NVIDIA Orin。_x000D_
-_x000D_
-3. 知识产权产出：预计 2 项发明专利（自适应 CFG + Safety-Guided FM）；论文投稿 NeurIPS/ICLR 级别顶会。_x000D_
-_x000D_
-4. 工程落地价值：三阶段渐进部署（影子模式 → 场景分级 → 最终替代），零风险落地；跨域迁移方案利用开源 nuPlan 数据预训练，少量公司数据微调即可适配。_x000D_
-_x000D_
-5. 技术延续性：从之前的「超让标签离散决策」升级为「连续轨迹端到端规划」，超让标签数据可直接复用为自适应 CFG 条件信号，与之前项目成果无缝衔接。</t>
+    <t>1. 基线复现与验证：Flow Planner 在 nuPlan Val14 达到 NR=90.43，超过 Diffusion Planner (89.87)
+2. Goal Point 体系搭建：64 类聚类 goal vocabulary (goal_vocab.npy)，基于 4s@10Hz 轨迹终点聚类
+3. Goal Conditioning 架构集成：goal_proj MLP + AdaLN 注入 decoder
+4. DPO Pipeline 完整实现：goal 聚类 → 候选生成 → 评分 → DPO 训练，端到端自动化脚本                6. 安全推理机制原型：best-of-N 筛选 + Risk-Adaptive ODE + TTC/DRAC 校验
+7. 技术文档与部署指南：，支持一键部署到训练服务器</t>
   </si>
   <si>
-    <t>1. 首次在 Flow Matching 框架中实现完整的安全自适应系统：现有 Flow Planner / Diffusion Planner 均使用固定引导参数和推理步数。本项目首次提出基于场景风险评估的自适应引导策略（Risk-Aware CFG）和动态推理精度控制（Risk-Adaptive ODE）。_x000D_
-_x000D_
-2. 首次将 DPO 偏好对齐应用于 Flow Matching 轨迹规划：借鉴 GoalFlow (CVPR 2025) 的 goal point conditioning 解决 FM 的模式坍塌问题，使 DPO 偏好学习在 Flow Matching 框架中首次可行。目前学界（TrajHF、MuDi-Pro）对轨迹偏好对齐刚起步。_x000D_
-_x000D_
-3. Safety-Guided Flow Matching 完全原创：现有安全引导工作（CATG、CGD）均基于 Diffusion 模型，本方案首次在 Flow Matching 的 ODE 求解过程中注入安全约束梯度，不改变模型结构、零额外训练成本。_x000D_
-_x000D_
-4. 与公司业务深度结合：直接服务于 ASW Planning 模块，三阶段部署方案已设计完成，超让标签数据可直接复用。_x000D_
-_x000D_
-5. 行业领先性：Flow Planner 是 NeurIPS 2025 纯学习方法 SOTA (Val14 NR=90.43)。我们在 SOTA 基础上进一步增强安全性和自适应能力，在学术和工程两个维度同时推进。</t>
+    <t>一阶段收益（仿真验证）：
+- 多模态生成能力：轨迹多样性提升 3-5 倍，解决模式坍塌问题
+- 偏好对齐能力：DPO 后模型按公司安全偏好输出轨迹，Val14 NR 预期 &gt; 91
+- VLM 评分创新：业界首个将多模态大模型用于轨迹偏好裁判的 pipeline
+- Scene-Adaptive CFG：零训练成本 NR +9 分（71.2% -&gt; 80.2%），已完成验证
+- 论文 1 篇 + 专利 1 项（VLM+DPO 偏好对齐方法）
+二阶段收益（实车部署）：
+- 跨域迁移：建立 nuPlan -&gt; 公司场景的完整迁移 pipeline（冻结浅层 + 微调 Decoder）
+- 部署能力：TensorRT FP16 .engine 文件 &lt;30MB，延迟 &lt;50ms，满足 10Hz 实时性
+- 渐进部署：影子模式 -&gt; 场景分级混合 -&gt; 全场景接管，风险可控
+- 产品价值：生成式候选适合博弈/多车交互场景，补充 rule-based planner 盲区
+- 可定制性：换打分标准重跑 DPO 即可适配不同客户/市场驾驶风格
+- 专利 2 项（自适应 CFG + Safety-Guided FM）+ 论文 1 篇
+战略收益：
+- 技术储备对标 Tesla FSD v12 / Waymo EMMA 的端到端生成式规划方向
+- 掌握 Flow Matching + Goal Conditioning + DPO 全链路 know-how
+- 专利总计 3 项，覆盖偏好对齐、自适应推理、安全引导三个核心创新方向</t>
   </si>
   <si>
-    <t>第一部分 (基线复现与算法创新): 第1月 - 第6月 (共6个月)_x000D_
-  - 第1-3月：nuPlan 全量数据预处理, Flow Planner 基线复现, 目标 Val14 NR &gt;= 90_x000D_
-  - 第4-6月：5大创新模块开发 + 消融实验 + Goal-Conditioned DPO Pipeline 搭建与验证_x000D_
-    目标: Val14 NR &gt; 91, InterPlan &gt; 65_x000D_
-_x000D_
-第二部分 (跨域迁移与实车验证): 第7月 - 第10月 (共4个月)_x000D_
-  - 第7-8月：公司数据格式适配 + 迁移训练 + TensorRT FP16 量化_x000D_
-    目标: 公司仿真闭环通过, 推理延迟 &lt; 50ms_x000D_
-  - 第9-10月：NVIDIA Orin 平台部署 + 实车路口场景调试 + 专利/论文撰写_x000D_
-    目标: 实车验证通过, 提交 2 项发明专利</t>
+    <t>一阶段：仿真验证（第1月 - 第6月）
+第1-2月：Goal Conditioning 微调与多模态生成验证
+  - 交付：goal-conditioned checkpoint + 多模态评估报告
+  - 指标：trajectory spread 提升 3x+，不同 goal 生成视觉可区分轨迹
+  - 资源：4x A100（AutoDL）
+第3-4月：Hybrid Scoring + DPO 偏好对齐
+  - 交付：DPO LoRA checkpoint + 消融实验报告 + 专利初稿（VLM+DPO 方法）
+  - 指标：Val14 NR &gt;= 91，chosen 安全性显著优于 rejected
+  - 资源：2x A100
+第5-6月：Safety-Aware Inference 集成 + 论文撰写
+  - 交付：完整推理 pipeline（Scene-Adaptive CFG + best-of-N + safety check）+ 论文初稿
+  - 指标：碰撞率降低 30%+，推理延迟 &lt; 50ms
+  - 资源：RTX 4090
+二阶段：实车部署（第7月 - 第12月）
+第7-8月：跨域迁移 + TensorRT 量化
+  - 交付：公司数据微调 checkpoint + TensorRT FP16 .engine 文件
+  - 方案：冻结 Encoder 浅层 + 微调 Decoder，适配公司传感器/场景分布
+  - 指标：模型 &lt;30MB，延迟 &lt;50ms，公司场景基础功能验证
+  - 资源：RTX 4090 + 公司数据接入
+第9-10月：三阶段部署执行
+  - 阶段 A - 影子模式：Flow Planner 与现有 planner 并行运行，采集对比数据
+  - 阶段 B - 场景分级混合：路口/博弈等复杂场景由 Flow Planner 接管
+  - 阶段 C - 全场景接管：全场景运行，rule-based 作为安全兜底
+  - 交付：影子模式对比报告 + 场景分级混合方案
+  - 资源：Orin 开发板 + 实车测试环境
+第11-12月：验收与结题
+  - 交付：实车验证报告（碰撞率/TTC 合规率/舒适度/通过率）+ 2 项专利提交 + 结题报告
+  - 指标：实车路口场景闭环测试通过
+  - 资源：实车测试 + 内部评审</t>
   </si>
   <si>
-    <t>算力支持 (High Priority):_x000D_
-a. 训练服务器：4x NVIDIA A100 (80GB) GPU, 约 2000-3000 卡时 (约 1-1.5 万元, AutoDL 云端)_x000D_
-b. 消融实验：2x A100, 约 800-1200 卡时 (约 0.4-0.6 万元)_x000D_
-c. 日常开发：RTX 4090, 约 1500 卡时 (约 0.3 万元)_x000D_
-d. 数据存储：AutoDL 数据盘 200GB (约 0.3 万元)_x000D_
-第一阶段小计：约 2-3 万元 (AutoDL 云端)_x000D_
-_x000D_
-开发人员:_x000D_
-a. 1 名算法工程师 (全职, 负责模型训练、创新模块开发、DPO Pipeline)_x000D_
-b. 使用 nuPlan 开源数据 (4城市 100万+ 场景), 无额外数据标注成本</t>
+    <t>二阶段资源（实车部署，M7-M12）：                            小计 ~7 万
+a. 跨域迁移训练算力
+   A100 / RTX 4090，公司数据微调多轮迭代 + TensorRT 量化调试   ~2.5 万
+b. NVIDIA Orin 开发板（含配件）                                ~1.0 万
+c. 实车测试费用
+   测试场地租用 + 车辆使用 + 安全员                            ~2.0 万
+d. 公司数据标注与预处理
+   内部数据团队协作 + 外包标注                                 ~1.0 万
+e. 备用算力（长尾场景补训 + 部署后在线微调实验）               ~0.5 万
+二阶段小计：~7.0 万</t>
   </si>
   <si>
-    <t>1. 基线模型：nuPlan 全量数据训练完成, Val14 NR &gt;= 90 (已完成: Open-Loop ADE=2.48m, FDE=5.73m, 超越官方权重 2-4%)_x000D_
-2. 创新模块代码：Scene-Adaptive CFG + Best-of-N + Risk-Adaptive ODE + Safety-Guided FM 完整实现_x000D_
-3. DPO Pipeline 代码：Goal 聚类 (cluster_goals.py) -&gt; 候选生成 (generate_candidates_goal.py) -&gt; 打分 (score_hybrid.py) -&gt; DPO 训练 (train_dpo.py) 端到端自动化 (已完成代码开发, 待部署验证)_x000D_
-4. Goal Vocabulary：64 个聚类中心 (goal_vocab.npy), 4s@10Hz 时间窗口_x000D_
-5. Bug 修复 13 处：collision detection, torch.norm 弃用, CFG argparse, encoder bugs 等_x000D_
-6. 消融实验报告：各创新模块的 NR Score / 碰撞率对比分析_x000D_
-7. 专利初稿：自适应 CFG 方法专利申请初稿</t>
+    <t xml:space="preserve">一阶段资源（仿真验证，M1-M6）：                            小计 ~8 万
+a. Goal Conditioning + DPO 多轮训练算力
+   4x A100 (80GB)，含 goal finetune、DPO、消融实验、重训      ~5.0 万
+b. 推理评估与 CFG Grid Search
+   RTX 4090，Val14 闭环评估、Scene-Adaptive CFG 全参数搜索     ~1.0 万
+c. VLM 评分 API 调用
+   Gemini API（BEV 图像 + 文本，约 5 万次调用）                ~1.0 万
+d. 数据存储与传输
+   AutoDL 云盘 500GB + nuPlan 数据下载带宽                     ~0.5 万
+一阶段小计：~8.0 万
+ </t>
   </si>
   <si>
-    <t>算力支持:_x000D_
-a. 公司内部 GPU 集群 (使用公司数据, 不可上传第三方平台, 必须内部 GPU)_x000D_
-b. 迁移训练 + 微调实验, 预计 GPU 占用约 4-6 周_x000D_
-c. 本地/车端计算平台 (NVIDIA Orin) 用于部署测试与实车验证_x000D_
+    <t>一阶段可期待交付物（仿真验证，M1-M6）：_x000D_
+1. 多模态轨迹生成模型：经 nuPlan Val14 验证的 Goal-Conditioned Flow Planner，同场景可生成 3+ 种决策级轨迹（左绕/右绕/刹停）_x000D_
+2. 偏好对齐训练 Pipeline：从候选生成、混合评分（规则 + VLM）、到 DPO 训练的端到端工具链，可复用于不同偏好标准_x000D_
+3. 仿真闭环验证报告：nuPlan Val14 全指标评估（NR &gt; 91、碰撞率、舒适度、轨迹多样性对比）_x000D_
+4. Scene-Adaptive CFG 技术验证报告：CFG 权重 grid search 实验数据、最优参数推荐、与 baseline 对比（NR +9 分）_x000D_
+5. 论文 1 篇（Goal-Conditioned DPO，投稿 NeurIPS/ICLR 2026）_x000D_
+6. 发明专利 1 项（VLM + DPO 轨迹偏好对齐方法）_x000D_
 _x000D_
-开发人员:_x000D_
-a. 算法工程师继续投入, 重点转向工程化部署与 TensorRT 优化_x000D_
-b. 需协调实车测试所需的车辆与场地资源_x000D_
-_x000D_
-第二阶段小计：公司内部资源 (需提前协调 GPU 配额与测试车辆)</t>
+二阶段可期待交付物（实车部署，M7-M12）：_x000D_
+1. 跨域迁移模型：nuPlan 预训练 -&gt; 公司数据微调的 Flow Planner（冻结 Encoder 浅层 + 微调 Decoder）_x000D_
+2. 车端部署模型：TensorRT FP16 量化后的 .engine 文件，推理延迟 &lt; 50ms，满足 10Hz 实时性_x000D_
+3. 三阶段部署方案：影子模式对比数据 + 场景分级混合部署方案 + 全场景接管方案_x000D_
+4. 实车验证报告：路口场景闭环测试结果（碰撞率、TTC 合规率、舒适度、通过率）_x000D_
+5. 发明专利 2 项正式提交（自适应 CFG + Safety-Guided Flow Matching）_x000D_
+6. 结题报告：完整技术方案、实验数据、部署方案、投入产出分析</t>
   </si>
   <si>
-    <t>1. 跨域迁移模型：nuPlan 预训练 -&gt; 公司数据微调的 Flow Planner 模型 (冻结 Encoder 浅层 + 微调 Decoder)_x000D_
-2. 车端部署模型：TensorRT FP16 量化后的 .engine 文件, 推理延迟 &lt; 50ms, 满足 10Hz 实时性_x000D_
-3. 三阶段部署执行：影子模式对比数据 + 场景分级混合部署方案 + 全场景接管方案_x000D_
-4. 实车验证报告：路口场景闭环测试结果 (碰撞率, TTC 合规率, 舒适度, 通过率)_x000D_
-5. 2 项发明专利正式提交 (自适应 CFG + Safety-Guided Flow Matching)_x000D_
-6. 结题报告：完整技术方案、实验数据、部署方案、投入产出分析</t>
+    <t>1. 多模态轨迹生成模型：经 nuPlan Val14 验证的 Goal-Conditioned Flow Planner，同场景可生成 3+ 种决策级轨迹（左绕/右绕/刹停）
+2. 偏好对齐训练 Pipeline：从候选生成、混合评分（规则 + VLM）、到 DPO 训练的端到端工具链，可复用于不同偏好标准
+3. 仿真闭环验证报告：nuPlan Val14 全指标评估（NR &gt; 91、碰撞率、舒适度、轨迹多样性对比）
+4. Scene-Adaptive CFG 技术验证报告：CFG 权重 grid search 实验数据、最优参数推荐、与 baseline 对比（NR +9 分）
+5. 论文 1 篇（Goal-Conditioned DPO，投稿 NeurIPS/ICLR 2026）
+6. 发明专利 1 项（VLM + DPO 轨迹偏好对齐方法）</t>
   </si>
 </sst>
 </file>
@@ -377,92 +406,3580 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>392206</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>22411</xdr:rowOff>
+      <xdr:colOff>227003</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>46028</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>171314</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>1102022</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>70919</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>1451283</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="4" name="组合 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{16D16CE0-741E-68BE-91FF-FB88E7B33F76}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6329B46-A922-2C89-D978-296FCDA65C42}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7877735" y="1725705"/>
-          <a:ext cx="10568692" cy="9637059"/>
+          <a:off x="7736167" y="1389919"/>
+          <a:ext cx="10054716" cy="7348855"/>
+          <a:chOff x="317500" y="1460500"/>
+          <a:chExt cx="10045700" cy="7327900"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>257733</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>561923</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>17664</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>98807</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="图片 1">
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="63" name="矩形 62">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BAAE33D6-6552-1DDF-FE30-24AEBE3265F4}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="317500" y="1460500"/>
+            <a:ext cx="10045700" cy="7327900"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:miter lim="800000"/>
+          </a:ln>
+          <a:effectLst/>
           <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBF45858-1EC2-33A8-6C54-7D65BA63FE61}"/>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a14:hiddenFill>
             </a:ext>
           </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7766897" y="2501559"/>
-          <a:ext cx="13541393" cy="10906459"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="en-US" sz="1100" kern="1200"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="2" name="矩形 1">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B27C9B6-4BC6-A204-1F14-0C6DBA7220E6}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="444500" y="1524000"/>
+            <a:ext cx="9410700" cy="355600"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+            <a:miter lim="800000"/>
+          </a:ln>
+          <a:effectLst/>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:shade val="15000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+                <a:miter lim="800000"/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Flow Planner </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="1400" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>自主驾驶研究项目</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1400" b="1" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="3" name="矩形 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ABE7AF0C-7536-21CB-353D-FA014BADCF57}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="444500" y="1968500"/>
+            <a:ext cx="2984500" cy="482600"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="E6E6E6"/>
+          </a:solidFill>
+          <a:ln w="22860">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>数据工程流水线 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Data Pipeline)</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="23" name="矩形 22">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62E07030-0712-293E-A2BE-332032CD6916}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3657600" y="1968500"/>
+            <a:ext cx="2984500" cy="482600"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="E6E6E6"/>
+          </a:solidFill>
+          <a:ln w="22860">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>基线与创新改进 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Model Innovation)</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="24" name="矩形 23">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C1D5A0A-B91F-3D0F-2507-15DAF28835E0}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6870700" y="1968500"/>
+            <a:ext cx="2984500" cy="482600"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="E6E6E6"/>
+          </a:solidFill>
+          <a:ln w="22860">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>训练与实车部署 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="900" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Training &amp; Deploy)</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="25" name="矩形: 圆角 24">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{039BD059-E3E0-8819-25F7-3D7E7889B6BB}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="444500" y="2552700"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>nuPlan</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>数据预处理 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Extraction)
+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>处理</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>4</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>城市</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>1500</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>h</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>驾驶数据，提取</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>ego/agent/map</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>特征，转为</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>npz</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>格式</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="26" name="直接连接符 25">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{426283AE-2B5E-EDD5-7E71-50787D67EB23}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1936750" y="3390900"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="27" name="矩形: 圆角 26">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BFE97C7-15E3-15D7-D321-0456F8A365A1}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="444500" y="3619500"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>坐标变换与归一化 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Alignment)
+ego-centric</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>前左上坐标系变换，静态统计量标准化</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="28" name="直接连接符 27">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B1DCA1A9-357C-CE6E-9F9F-7D46ADCE2F60}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1936750" y="4457700"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="29" name="矩形: 圆角 28">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E19FB4B-E374-A1D9-723B-20343DE65328}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="444500" y="4686300"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>GT</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>轨迹终点聚类 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Goal Clustering)
+4s@10Hz</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>轨迹终点，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>K-Means K=64，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>构建</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>goal_vocab.npy</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="30" name="直接连接符 29">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94D3AAE8-B83B-C07E-694A-802EAFA68E7A}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1936750" y="5524500"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="31" name="矩形: 圆角 30">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98F88BD4-EBCF-5932-D346-AD4D11F688F0}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="444500" y="5753100"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>数据增强 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Augmentation)
+ego</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>状态随机扰动</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>五次多模式轨迹插值，提升闭环鲁棒性</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="32" name="直接连接符 31">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11139F53-25CA-3F27-C67D-48BAA738C8F3}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1936750" y="6591300"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="33" name="矩形: 圆角 32">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7EC3B0A9-0189-FDC2-6D5C-14888346308D}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="444500" y="6819900"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>公司数据适配 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Domain Adaptation)
+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>公司内部数据预处理，传感器</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>/</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>坐标系</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>/</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>场景分布对齐，跨域迁移</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="34" name="矩形: 圆角 33">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9CEC5E3-A4D3-B319-BA5A-AEBDF417420C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3657600" y="2552700"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>搭建</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Flow Planner</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>基线 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Baseline)
+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>复现</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>MLP-Mixer Encoder + DiT Decoder + Flow Matching ODE</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="35" name="直接连接符 34">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{351F71C2-D8CD-AA94-483C-B5FA588B5EA6}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5149850" y="3390900"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="36" name="菱形 35">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0532152E-7922-EDA2-0018-B1DFA07879C9}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3784600" y="3619500"/>
+            <a:ext cx="2730500" cy="711200"/>
+          </a:xfrm>
+          <a:prstGeom prst="diamond">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFDC"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="228600" rIns="228600" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>判定：</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Val14 NR&gt;=90?
+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>确认基线达到论文</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>SOTA</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>水平</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="750" b="1" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="37" name="矩形 36">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A73D1C8-E8ED-81BF-B55A-10DCB6C72924}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6540500" y="3886200"/>
+            <a:ext cx="304800" cy="177800"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+            <a:miter lim="800000"/>
+          </a:ln>
+          <a:effectLst/>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:shade val="15000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+                <a:miter lim="800000"/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="C80000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>no</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="38" name="矩形 37">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0D62209-0B90-4845-A7D7-CF91804DF96F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="4997450" y="4343400"/>
+            <a:ext cx="304800" cy="177800"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+            <a:miter lim="800000"/>
+          </a:ln>
+          <a:effectLst/>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:shade val="15000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+                <a:miter lim="800000"/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="007800"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>yes</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="39" name="直接连接符 38">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B1F21FE0-A663-9392-1F6F-9906C3B4BB0D}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5149850" y="4330700"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="40" name="矩形: 圆角 39">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02BE8B45-65B0-A1BA-DB30-701E8FFAAA4F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3657600" y="4559300"/>
+            <a:ext cx="2984500" cy="965200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="EBF5FF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>创新点</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>1</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>：</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Goal-Conditioned</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>意图注入
+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>64</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>个</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>goal point</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>通过</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>goal_proj MLP+AdaLN</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>注入</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Decoder，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>实现左绕</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>/</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>右绕</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>/</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>刹停等多模态轨迹生成</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="41" name="直接连接符 40">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8CB9EF4-1155-A9D5-6E8F-C1E6F164C4F7}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5149850" y="5524500"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="42" name="矩形: 圆角 41">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBE024AD-7589-B4E9-B05A-EFBEAFDEB7A1}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3657600" y="5753100"/>
+            <a:ext cx="2984500" cy="965200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="EBF5FF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>创新点</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>2</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>：</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>DPO</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>偏好对齐 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Preference)
+Scorer</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>多维评分构造</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>chosen/rejected</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>对，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>LoRA+DPO</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>微调，学习公司驾驶偏好</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="43" name="直接连接符 42">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBA11C19-75C5-87BB-F46D-9430C07418A5}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="5149850" y="6718300"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="44" name="矩形: 圆角 43">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDBF8A71-9017-37C4-F48D-C5B2C21ED2AB}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3657600" y="6946900"/>
+            <a:ext cx="2984500" cy="965200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="EBF5FF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>创新点</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>3</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>：</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Safety-Aware Inference
+TTC/DRAC</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>碰撞校验</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Best-of-N</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>筛选</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Adaptive ODE，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>安全推理兜底机制</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="45" name="矩形: 圆角 44">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1236FCD-08D0-1FAE-ECE1-BEAFC0CD2249}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6870700" y="2552700"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Goal-Conditioned Finetune
+Flow ODE+Goal Conditioning</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>训练，验证多模态生成，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>30% </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>CFG</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>掩码</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="46" name="直接连接符 45">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6AB20619-89C9-54C9-2BF5-E7B6A42A42D6}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8362950" y="3390900"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="47" name="矩形: 圆角 46">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AF1F670-72F2-3A27-9F96-2A7130A0F942}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6870700" y="3619500"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>DPO</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>训练与消融评测 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Testing)
+Goal</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>消融</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>/</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>DPO</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>消融</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>/</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Safety</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>消融，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Val14+InterPlan</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>闭环仿真</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="48" name="直接连接符 47">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{983B5764-F34A-E868-5D26-FF3B117E0F4D}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8362950" y="4457700"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="49" name="菱形 48">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2AE5853-DD44-19A5-5D1D-54BC7D185ACA}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6997700" y="4686300"/>
+            <a:ext cx="2730500" cy="711200"/>
+          </a:xfrm>
+          <a:prstGeom prst="diamond">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFDC"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="228600" rIns="228600" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>判定：性能与效率达标</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>?
+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>NR&gt;91, InterPlan&gt;65, &lt;50ms</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="50" name="矩形 49">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E1119F9-D021-8958-BAE7-79B59859BCC0}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="9753600" y="4953000"/>
+            <a:ext cx="304800" cy="177800"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+            <a:miter lim="800000"/>
+          </a:ln>
+          <a:effectLst/>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:shade val="15000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+                <a:miter lim="800000"/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="C80000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>no</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="51" name="直接连接符 50">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA37FF8E-6F5D-9D17-4879-0751C9D40389}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="9728200" y="5041900"/>
+            <a:ext cx="355600" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="15240">
+            <a:solidFill>
+              <a:srgbClr val="333333"/>
+            </a:solidFill>
+            <a:prstDash val="dash"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="52" name="直接连接符 51">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CFA1ED3E-742F-3ABB-2AE7-CD5372D76690}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10083800" y="2971800"/>
+            <a:ext cx="0" cy="2070100"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="15240">
+            <a:solidFill>
+              <a:srgbClr val="333333"/>
+            </a:solidFill>
+            <a:prstDash val="dash"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="53" name="直接连接符 52">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7538A12A-FB0D-1CED-A021-84BF3597C942}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipH="1">
+            <a:off x="9855200" y="2971800"/>
+            <a:ext cx="228600" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="15240">
+            <a:solidFill>
+              <a:srgbClr val="333333"/>
+            </a:solidFill>
+            <a:prstDash val="dash"/>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="54" name="矩形 53">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B92BB49-AEFC-5B58-A6CF-99D5E5050BD2}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8210550" y="5410200"/>
+            <a:ext cx="304800" cy="177800"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+            <a:miter lim="800000"/>
+          </a:ln>
+          <a:effectLst/>
+          <a:extLst>
+            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a14:hiddenFill>
+            </a:ext>
+            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:shade val="15000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+                <a:miter lim="800000"/>
+              </a14:hiddenLine>
+            </a:ext>
+          </a:extLst>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="750" b="1" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="007800"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>yes</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="55" name="直接连接符 54">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{50F48F1A-E35B-1A48-D0C6-33A003A70B45}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8362950" y="5397500"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="56" name="矩形: 圆角 55">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADE74AA4-C0A1-A68C-34EC-DB3E800011A1}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6870700" y="5626100"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>TensorRT</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>量化与剪枝 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Optimization)
+FP16/INT8</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>量化，结构剪枝，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Batch Inference</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>并行加速</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="57" name="直接连接符 56">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DB9D11A-7776-7DE2-1C3B-BD52B7C5640A}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8362950" y="6464300"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="58" name="矩形: 圆角 57">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CCA3CBA-39A4-A520-4EF2-84CB2B3AB5E6}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6870700" y="6692900"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>公司数据训练与验证
+公司内部数据集微调，闭环仿真验证，适配公司场景分布</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="59" name="直接连接符 58">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4020C9A-7C8F-94FA-758F-DE4AAA7CD60B}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="8362950" y="7531100"/>
+            <a:ext cx="0" cy="228600"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="60" name="矩形: 圆角 59">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B7E258B-4108-4E1B-F310-53C89F9B260F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6870700" y="7759700"/>
+            <a:ext cx="2984500" cy="838200"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="76200" tIns="38100" rIns="76200" bIns="38100" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>实车调试与部署 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Vehicle Testing)
+</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>部署至</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>NVIDIA Orin，</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>接入</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>Planning</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="zh-CN" altLang="en-US" sz="800" kern="1200">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+              </a:rPr>
+              <a:t>闭环，实车路口场景验证</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="800" kern="1200">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Microsoft YaHei UI" panose="020B0503020204020204" pitchFamily="34" charset="-122"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="61" name="直接连接符 60">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E48D3195-07C9-B998-62F6-1C9C56190C2D}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3429000" y="2971800"/>
+            <a:ext cx="228600" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="62" name="直接连接符 61">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{835C79A5-3CF8-B6B7-A904-E5670B19B0B5}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6642100" y="2971800"/>
+            <a:ext cx="228600" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="line">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -821,7 +4338,7 @@
     <row r="14" spans="1:30" ht="59.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
@@ -858,7 +4375,7 @@
     <row r="17" spans="1:30" ht="165.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="B17" s="13" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
@@ -894,7 +4411,7 @@
     <row r="20" spans="1:30" ht="205.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
       <c r="B20" s="14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
@@ -920,7 +4437,7 @@
     <row r="23" spans="1:30" ht="129" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C23" s="11"/>
       <c r="D23" s="11"/>
@@ -946,7 +4463,7 @@
     <row r="26" spans="1:30" ht="70.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8"/>
       <c r="B26" s="10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
@@ -998,7 +4515,7 @@
     <row r="32" spans="1:30" ht="183" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8"/>
       <c r="B32" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
@@ -1024,7 +4541,7 @@
     <row r="35" spans="1:11" ht="133.19999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
       <c r="B35" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
@@ -1047,7 +4564,7 @@
     <row r="38" spans="1:11" ht="183" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8"/>
       <c r="B38" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
@@ -1073,7 +4590,7 @@
     <row r="41" spans="1:11" ht="133.19999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8"/>
       <c r="B41" s="10" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C41" s="11"/>
       <c r="D41" s="11"/>

</xml_diff>